<commit_message>
remove Reversal contrast from pilot
</commit_message>
<xml_diff>
--- a/04_Figures/F04/c_data/F04_supplementary.xlsx
+++ b/04_Figures/F04/c_data/F04_supplementary.xlsx
@@ -41574,25 +41574,25 @@
         <v>257</v>
       </c>
       <c r="D2" t="n">
-        <v>3.48412721247144</v>
+        <v>3.48412721247087</v>
       </c>
       <c r="E2" t="n">
-        <v>4.21161096897943</v>
+        <v>4.21161096897874</v>
       </c>
       <c r="F2" t="n">
-        <v>0.511141040596112</v>
+        <v>0.511141040596108</v>
       </c>
       <c r="G2" t="n">
-        <v>0.556196949731643</v>
+        <v>0.556196949731639</v>
       </c>
       <c r="H2" t="n">
-        <v>0.0287632004854426</v>
+        <v>0.0287632004854827</v>
       </c>
       <c r="I2" t="s">
         <v>258</v>
       </c>
       <c r="J2" t="n">
-        <v>4.21161096897943</v>
+        <v>4.21161096897874</v>
       </c>
       <c r="K2" t="s">
         <v>53</v>
@@ -41609,25 +41609,25 @@
         <v>257</v>
       </c>
       <c r="D3" t="n">
-        <v>4.05790561093459</v>
+        <v>4.0579056109332</v>
       </c>
       <c r="E3" t="n">
-        <v>4.09186896159811</v>
+        <v>4.09186896159673</v>
       </c>
       <c r="F3" t="n">
         <v>0.706915668807515</v>
       </c>
       <c r="G3" t="n">
-        <v>0.647715157272707</v>
+        <v>0.64771515727271</v>
       </c>
       <c r="H3" t="n">
-        <v>0.0021342337189146</v>
+        <v>0.00213423371892398</v>
       </c>
       <c r="I3" t="s">
         <v>258</v>
       </c>
       <c r="J3" t="n">
-        <v>4.09186896159811</v>
+        <v>4.09186896159673</v>
       </c>
       <c r="K3" t="s">
         <v>53</v>
@@ -41644,25 +41644,25 @@
         <v>259</v>
       </c>
       <c r="D4" t="n">
-        <v>-3.48817220034395</v>
+        <v>-3.48817220034216</v>
       </c>
       <c r="E4" t="n">
-        <v>-3.45429041055526</v>
+        <v>-3.45429041055345</v>
       </c>
       <c r="F4" t="n">
         <v>-0.764142564725145</v>
       </c>
       <c r="G4" t="n">
-        <v>-0.739464072659473</v>
+        <v>-0.739464072659466</v>
       </c>
       <c r="H4" t="n">
-        <v>0.00480638078838086</v>
+        <v>0.00480638078840438</v>
       </c>
       <c r="I4" t="s">
         <v>260</v>
       </c>
       <c r="J4" t="n">
-        <v>3.45429041055526</v>
+        <v>3.45429041055345</v>
       </c>
       <c r="K4" t="s">
         <v>77</v>
@@ -41679,10 +41679,10 @@
         <v>257</v>
       </c>
       <c r="D5" t="n">
-        <v>2.59704840828352</v>
+        <v>2.59704840828154</v>
       </c>
       <c r="E5" t="n">
-        <v>3.4307237061489</v>
+        <v>3.43072370614627</v>
       </c>
       <c r="F5" t="n">
         <v>1.10652955402938</v>
@@ -41691,13 +41691,13 @@
         <v>1.71883830144357</v>
       </c>
       <c r="H5" t="n">
-        <v>0.00758883678458743</v>
+        <v>0.00758883678463336</v>
       </c>
       <c r="I5" t="s">
         <v>258</v>
       </c>
       <c r="J5" t="n">
-        <v>3.4307237061489</v>
+        <v>3.43072370614627</v>
       </c>
       <c r="K5" t="s">
         <v>53</v>
@@ -41714,25 +41714,25 @@
         <v>259</v>
       </c>
       <c r="D6" t="n">
-        <v>-4.64310062264202</v>
+        <v>-4.6431006226428</v>
       </c>
       <c r="E6" t="n">
-        <v>-2.91801758322947</v>
+        <v>-2.91801758322992</v>
       </c>
       <c r="F6" t="n">
         <v>-0.481424194198407</v>
       </c>
       <c r="G6" t="n">
-        <v>-0.309755822129897</v>
+        <v>-0.309755822129894</v>
       </c>
       <c r="H6" t="n">
-        <v>0.00523848038285882</v>
+        <v>0.00523848038285669</v>
       </c>
       <c r="I6" t="s">
         <v>260</v>
       </c>
       <c r="J6" t="n">
-        <v>2.91801758322947</v>
+        <v>2.91801758322992</v>
       </c>
       <c r="K6" t="s">
         <v>77</v>
@@ -41749,25 +41749,25 @@
         <v>257</v>
       </c>
       <c r="D7" t="n">
-        <v>3.76368067195969</v>
+        <v>3.7636806719603</v>
       </c>
       <c r="E7" t="n">
-        <v>2.88994882485847</v>
+        <v>2.88994882485898</v>
       </c>
       <c r="F7" t="n">
         <v>0.390491085452169</v>
       </c>
       <c r="G7" t="n">
-        <v>0.306973060642736</v>
+        <v>0.30697306064274</v>
       </c>
       <c r="H7" t="n">
-        <v>0.0458883291390347</v>
+        <v>0.0458883291390167</v>
       </c>
       <c r="I7" t="s">
         <v>258</v>
       </c>
       <c r="J7" t="n">
-        <v>2.88994882485847</v>
+        <v>2.88994882485898</v>
       </c>
       <c r="K7" t="s">
         <v>53</v>
@@ -41784,25 +41784,25 @@
         <v>257</v>
       </c>
       <c r="D8" t="n">
-        <v>4.63625010648219</v>
+        <v>4.63625010648508</v>
       </c>
       <c r="E8" t="n">
-        <v>2.88766399959163</v>
+        <v>2.88766399959336</v>
       </c>
       <c r="F8" t="n">
-        <v>0.433831594366467</v>
+        <v>0.43383159436647</v>
       </c>
       <c r="G8" t="n">
-        <v>0.25369598668917</v>
+        <v>0.253695986689166</v>
       </c>
       <c r="H8" t="n">
-        <v>0.00936752333387038</v>
+        <v>0.00936752333383787</v>
       </c>
       <c r="I8" t="s">
         <v>258</v>
       </c>
       <c r="J8" t="n">
-        <v>2.88766399959163</v>
+        <v>2.88766399959336</v>
       </c>
       <c r="K8" t="s">
         <v>53</v>
@@ -41819,25 +41819,25 @@
         <v>257</v>
       </c>
       <c r="D9" t="n">
-        <v>5.39120431822511</v>
+        <v>5.39120431822785</v>
       </c>
       <c r="E9" t="n">
-        <v>2.75946428310905</v>
+        <v>2.75946428311049</v>
       </c>
       <c r="F9" t="n">
         <v>0.473425956401499</v>
       </c>
       <c r="G9" t="n">
-        <v>0.248086314903819</v>
+        <v>0.248086314903823</v>
       </c>
       <c r="H9" t="n">
-        <v>0.00154451475019756</v>
+        <v>0.00154451475019221</v>
       </c>
       <c r="I9" t="s">
         <v>258</v>
       </c>
       <c r="J9" t="n">
-        <v>2.75946428310905</v>
+        <v>2.75946428311049</v>
       </c>
       <c r="K9" t="s">
         <v>53</v>
@@ -41854,25 +41854,25 @@
         <v>259</v>
       </c>
       <c r="D10" t="n">
-        <v>-3.2056473247244</v>
+        <v>-3.2056473247226</v>
       </c>
       <c r="E10" t="n">
-        <v>-2.70712786773506</v>
+        <v>-2.70712786773349</v>
       </c>
       <c r="F10" t="n">
         <v>-0.814653105627791</v>
       </c>
       <c r="G10" t="n">
-        <v>-0.693627278270903</v>
+        <v>-0.693627278270892</v>
       </c>
       <c r="H10" t="n">
-        <v>0.00669950361201134</v>
+        <v>0.0066995036120439</v>
       </c>
       <c r="I10" t="s">
         <v>260</v>
       </c>
       <c r="J10" t="n">
-        <v>2.70712786773506</v>
+        <v>2.70712786773349</v>
       </c>
       <c r="K10" t="s">
         <v>77</v>
@@ -41889,10 +41889,10 @@
         <v>257</v>
       </c>
       <c r="D11" t="n">
-        <v>4.62111071584486</v>
+        <v>4.62111071584234</v>
       </c>
       <c r="E11" t="n">
-        <v>2.67928195405195</v>
+        <v>2.67928195405049</v>
       </c>
       <c r="F11" t="n">
         <v>1.11357792651978</v>
@@ -41901,13 +41901,13 @@
         <v>0.661004499617025</v>
       </c>
       <c r="H11" t="n">
-        <v>0.00000578698121708469</v>
+        <v>0.00000578698121715527</v>
       </c>
       <c r="I11" t="s">
         <v>258</v>
       </c>
       <c r="J11" t="n">
-        <v>2.67928195405195</v>
+        <v>2.67928195405049</v>
       </c>
       <c r="K11" t="s">
         <v>53</v>
@@ -41924,10 +41924,10 @@
         <v>259</v>
       </c>
       <c r="D12" t="n">
-        <v>-2.91392784946546</v>
+        <v>-2.91392784946407</v>
       </c>
       <c r="E12" t="n">
-        <v>-2.46744007168066</v>
+        <v>-2.46744007167948</v>
       </c>
       <c r="F12" t="n">
         <v>-0.608293578130187</v>
@@ -41936,13 +41936,13 @@
         <v>-0.441667173414015</v>
       </c>
       <c r="H12" t="n">
-        <v>0.0423994348400066</v>
+        <v>0.0423994348401228</v>
       </c>
       <c r="I12" t="s">
         <v>260</v>
       </c>
       <c r="J12" t="n">
-        <v>2.46744007168066</v>
+        <v>2.46744007167948</v>
       </c>
       <c r="K12" t="s">
         <v>77</v>
@@ -41959,10 +41959,10 @@
         <v>257</v>
       </c>
       <c r="D13" t="n">
-        <v>3.56494917113652</v>
+        <v>3.56494917113547</v>
       </c>
       <c r="E13" t="n">
-        <v>2.43367358253559</v>
+        <v>2.43367358253488</v>
       </c>
       <c r="F13" t="n">
         <v>0.538929847075671</v>
@@ -41971,13 +41971,13 @@
         <v>0.376663015654117</v>
       </c>
       <c r="H13" t="n">
-        <v>0.0200502138750866</v>
+        <v>0.0200502138751314</v>
       </c>
       <c r="I13" t="s">
         <v>258</v>
       </c>
       <c r="J13" t="n">
-        <v>2.43367358253559</v>
+        <v>2.43367358253488</v>
       </c>
       <c r="K13" t="s">
         <v>53</v>
@@ -41994,25 +41994,25 @@
         <v>259</v>
       </c>
       <c r="D14" t="n">
-        <v>-4.18249954175652</v>
+        <v>-4.18249954175475</v>
       </c>
       <c r="E14" t="n">
-        <v>-2.37026507714477</v>
+        <v>-2.37026507714375</v>
       </c>
       <c r="F14" t="n">
         <v>-0.769667406399485</v>
       </c>
       <c r="G14" t="n">
-        <v>-0.431402455948795</v>
+        <v>-0.431402455948792</v>
       </c>
       <c r="H14" t="n">
-        <v>0.000803919817790013</v>
+        <v>0.000803919817794644</v>
       </c>
       <c r="I14" t="s">
         <v>260</v>
       </c>
       <c r="J14" t="n">
-        <v>2.37026507714477</v>
+        <v>2.37026507714375</v>
       </c>
       <c r="K14" t="s">
         <v>77</v>
@@ -42029,25 +42029,25 @@
         <v>257</v>
       </c>
       <c r="D15" t="n">
-        <v>3.25356019722984</v>
+        <v>3.25356019722794</v>
       </c>
       <c r="E15" t="n">
-        <v>2.32286999909673</v>
+        <v>2.32286999909538</v>
       </c>
       <c r="F15" t="n">
         <v>0.900404254930402</v>
       </c>
       <c r="G15" t="n">
-        <v>0.413709003406984</v>
+        <v>0.413709003406986</v>
       </c>
       <c r="H15" t="n">
-        <v>0.00466372750745126</v>
+        <v>0.00466372750748004</v>
       </c>
       <c r="I15" t="s">
         <v>258</v>
       </c>
       <c r="J15" t="n">
-        <v>2.32286999909673</v>
+        <v>2.32286999909538</v>
       </c>
       <c r="K15" t="s">
         <v>53</v>
@@ -42064,25 +42064,25 @@
         <v>257</v>
       </c>
       <c r="D16" t="n">
-        <v>4.01785730469738</v>
+        <v>4.01785730469829</v>
       </c>
       <c r="E16" t="n">
-        <v>2.29300875076177</v>
+        <v>2.29300875076236</v>
       </c>
       <c r="F16" t="n">
         <v>0.402624473620964</v>
       </c>
       <c r="G16" t="n">
-        <v>0.235246478227097</v>
+        <v>0.235246478227104</v>
       </c>
       <c r="H16" t="n">
-        <v>0.0297225836246326</v>
+        <v>0.0297225836246106</v>
       </c>
       <c r="I16" t="s">
         <v>258</v>
       </c>
       <c r="J16" t="n">
-        <v>2.29300875076177</v>
+        <v>2.29300875076236</v>
       </c>
       <c r="K16" t="s">
         <v>53</v>
@@ -42099,25 +42099,25 @@
         <v>257</v>
       </c>
       <c r="D17" t="n">
-        <v>3.98464356645327</v>
+        <v>3.98464356645527</v>
       </c>
       <c r="E17" t="n">
-        <v>2.258562043822</v>
+        <v>2.25856204382324</v>
       </c>
       <c r="F17" t="n">
-        <v>0.349460320731538</v>
+        <v>0.349460320731534</v>
       </c>
       <c r="G17" t="n">
-        <v>0.2027926331901</v>
+        <v>0.202792633190107</v>
       </c>
       <c r="H17" t="n">
-        <v>0.0491609257512685</v>
+        <v>0.0491609257511754</v>
       </c>
       <c r="I17" t="s">
         <v>258</v>
       </c>
       <c r="J17" t="n">
-        <v>2.258562043822</v>
+        <v>2.25856204382324</v>
       </c>
       <c r="K17" t="s">
         <v>53</v>
@@ -42134,10 +42134,10 @@
         <v>257</v>
       </c>
       <c r="D18" t="n">
-        <v>3.73354463132608</v>
+        <v>3.73354463132412</v>
       </c>
       <c r="E18" t="n">
-        <v>2.13914502585512</v>
+        <v>2.139145025854</v>
       </c>
       <c r="F18" t="n">
         <v>0.776205944356491</v>
@@ -42146,13 +42146,13 @@
         <v>0.452181538535665</v>
       </c>
       <c r="H18" t="n">
-        <v>0.00257723117456075</v>
+        <v>0.00257723117457561</v>
       </c>
       <c r="I18" t="s">
         <v>258</v>
       </c>
       <c r="J18" t="n">
-        <v>2.13914502585512</v>
+        <v>2.139145025854</v>
       </c>
       <c r="K18" t="s">
         <v>53</v>
@@ -42169,10 +42169,10 @@
         <v>257</v>
       </c>
       <c r="D19" t="n">
-        <v>3.90789142328878</v>
+        <v>3.90789142328785</v>
       </c>
       <c r="E19" t="n">
-        <v>2.02585547110816</v>
+        <v>2.02585547110767</v>
       </c>
       <c r="F19" t="n">
         <v>0.611262057913592</v>
@@ -42181,13 +42181,13 @@
         <v>0.285039023149753</v>
       </c>
       <c r="H19" t="n">
-        <v>0.00639334703822229</v>
+        <v>0.00639334703823942</v>
       </c>
       <c r="I19" t="s">
         <v>258</v>
       </c>
       <c r="J19" t="n">
-        <v>2.02585547110816</v>
+        <v>2.02585547110767</v>
       </c>
       <c r="K19" t="s">
         <v>53</v>
@@ -42204,25 +42204,25 @@
         <v>257</v>
       </c>
       <c r="D20" t="n">
-        <v>4.63999909161891</v>
+        <v>4.63999909161652</v>
       </c>
       <c r="E20" t="n">
-        <v>1.95027028471477</v>
+        <v>1.95027028471379</v>
       </c>
       <c r="F20" t="n">
         <v>1.01770635395491</v>
       </c>
       <c r="G20" t="n">
-        <v>0.437936508011408</v>
+        <v>0.437936508011411</v>
       </c>
       <c r="H20" t="n">
-        <v>0.0000152558240329483</v>
+        <v>0.000015255824033112</v>
       </c>
       <c r="I20" t="s">
         <v>258</v>
       </c>
       <c r="J20" t="n">
-        <v>1.95027028471477</v>
+        <v>1.95027028471379</v>
       </c>
       <c r="K20" t="s">
         <v>53</v>
@@ -42239,10 +42239,10 @@
         <v>257</v>
       </c>
       <c r="D21" t="n">
-        <v>4.98144460589364</v>
+        <v>4.98144460589408</v>
       </c>
       <c r="E21" t="n">
-        <v>1.94065606360787</v>
+        <v>1.94065606360804</v>
       </c>
       <c r="F21" t="n">
         <v>0.540644965102562</v>
@@ -42251,13 +42251,13 @@
         <v>0.215633974661486</v>
       </c>
       <c r="H21" t="n">
-        <v>0.0014107092744133</v>
+        <v>0.0014107092744139</v>
       </c>
       <c r="I21" t="s">
         <v>258</v>
       </c>
       <c r="J21" t="n">
-        <v>1.94065606360787</v>
+        <v>1.94065606360804</v>
       </c>
       <c r="K21" t="s">
         <v>53</v>

</xml_diff>

<commit_message>
Refine F04 panel B layout
- widen F04 heatmap left (TILE_W 0.833, x_sig 0.27 via new cfg knobs;
  right edge anchored at HEAT_RIGHT)
- fill F04 bar plot to X_BAR_MAX (bar_scale 0.46, bar_ref_width 14)
- extend pathway row bg stripes to right edge (engine; affects F04 + F05)
- F05 panel B bottom margin 4mm -> 8mm for breathing room
</commit_message>
<xml_diff>
--- a/04_Figures/F04/c_data/F04_supplementary.xlsx
+++ b/04_Figures/F04/c_data/F04_supplementary.xlsx
@@ -46096,7 +46096,7 @@
         <v>3.3</v>
       </c>
       <c r="E2" t="n">
-        <v>4.82</v>
+        <v>4.1</v>
       </c>
     </row>
     <row r="3">
@@ -46110,10 +46110,10 @@
         <v>3</v>
       </c>
       <c r="D3" t="n">
-        <v>4.82</v>
+        <v>4.1</v>
       </c>
       <c r="E3" t="n">
-        <v>5.96</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="4">
@@ -46127,10 +46127,10 @@
         <v>1</v>
       </c>
       <c r="D4" t="n">
-        <v>5.96</v>
+        <v>4.7</v>
       </c>
       <c r="E4" t="n">
-        <v>6.34</v>
+        <v>4.9</v>
       </c>
     </row>
     <row r="5">
@@ -46147,7 +46147,7 @@
         <v>3.3</v>
       </c>
       <c r="E5" t="n">
-        <v>4.82</v>
+        <v>4.1</v>
       </c>
     </row>
     <row r="6">
@@ -46161,10 +46161,10 @@
         <v>2</v>
       </c>
       <c r="D6" t="n">
-        <v>4.82</v>
+        <v>4.1</v>
       </c>
       <c r="E6" t="n">
-        <v>5.58</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="7">
@@ -46178,10 +46178,10 @@
         <v>1</v>
       </c>
       <c r="D7" t="n">
-        <v>5.58</v>
+        <v>4.5</v>
       </c>
       <c r="E7" t="n">
-        <v>5.96</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="8">
@@ -46198,7 +46198,7 @@
         <v>3.3</v>
       </c>
       <c r="E8" t="n">
-        <v>4.06</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="9">
@@ -46212,10 +46212,10 @@
         <v>2</v>
       </c>
       <c r="D9" t="n">
-        <v>4.06</v>
+        <v>3.7</v>
       </c>
       <c r="E9" t="n">
-        <v>4.82</v>
+        <v>4.1</v>
       </c>
     </row>
     <row r="10">
@@ -46229,10 +46229,10 @@
         <v>1</v>
       </c>
       <c r="D10" t="n">
-        <v>4.82</v>
+        <v>4.1</v>
       </c>
       <c r="E10" t="n">
-        <v>5.2</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="11">
@@ -46249,7 +46249,7 @@
         <v>3.3</v>
       </c>
       <c r="E11" t="n">
-        <v>5.2</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="12">
@@ -46263,10 +46263,10 @@
         <v>2</v>
       </c>
       <c r="D12" t="n">
-        <v>5.2</v>
+        <v>4.3</v>
       </c>
       <c r="E12" t="n">
-        <v>5.96</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="13">
@@ -46280,10 +46280,10 @@
         <v>1</v>
       </c>
       <c r="D13" t="n">
-        <v>5.96</v>
+        <v>4.7</v>
       </c>
       <c r="E13" t="n">
-        <v>6.34</v>
+        <v>4.9</v>
       </c>
     </row>
     <row r="14">
@@ -46300,7 +46300,7 @@
         <v>3.3</v>
       </c>
       <c r="E14" t="n">
-        <v>5.2</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="15">
@@ -46314,10 +46314,10 @@
         <v>3</v>
       </c>
       <c r="D15" t="n">
-        <v>5.2</v>
+        <v>4.3</v>
       </c>
       <c r="E15" t="n">
-        <v>6.34</v>
+        <v>4.9</v>
       </c>
     </row>
     <row r="16">
@@ -46331,10 +46331,10 @@
         <v>2</v>
       </c>
       <c r="D16" t="n">
-        <v>6.34</v>
+        <v>4.9</v>
       </c>
       <c r="E16" t="n">
-        <v>7.1</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="17">
@@ -46351,7 +46351,7 @@
         <v>3.3</v>
       </c>
       <c r="E17" t="n">
-        <v>3.68</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="18">
@@ -46365,10 +46365,10 @@
         <v>1</v>
       </c>
       <c r="D18" t="n">
-        <v>3.68</v>
+        <v>3.5</v>
       </c>
       <c r="E18" t="n">
-        <v>4.06</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="19">
@@ -46382,10 +46382,10 @@
         <v>1</v>
       </c>
       <c r="D19" t="n">
-        <v>4.06</v>
+        <v>3.7</v>
       </c>
       <c r="E19" t="n">
-        <v>4.44</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="20">
@@ -46402,7 +46402,7 @@
         <v>3.3</v>
       </c>
       <c r="E20" t="n">
-        <v>5.2</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="21">
@@ -46416,10 +46416,10 @@
         <v>3</v>
       </c>
       <c r="D21" t="n">
-        <v>5.2</v>
+        <v>4.3</v>
       </c>
       <c r="E21" t="n">
-        <v>6.34</v>
+        <v>4.9</v>
       </c>
     </row>
     <row r="22">
@@ -46433,10 +46433,10 @@
         <v>1</v>
       </c>
       <c r="D22" t="n">
-        <v>6.34</v>
+        <v>4.9</v>
       </c>
       <c r="E22" t="n">
-        <v>6.72</v>
+        <v>5.1</v>
       </c>
     </row>
     <row r="23">
@@ -46453,7 +46453,7 @@
         <v>3.3</v>
       </c>
       <c r="E23" t="n">
-        <v>4.44</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="24">
@@ -46467,10 +46467,10 @@
         <v>3</v>
       </c>
       <c r="D24" t="n">
-        <v>4.44</v>
+        <v>3.9</v>
       </c>
       <c r="E24" t="n">
-        <v>5.58</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="25">
@@ -46484,10 +46484,10 @@
         <v>1</v>
       </c>
       <c r="D25" t="n">
-        <v>5.58</v>
+        <v>4.5</v>
       </c>
       <c r="E25" t="n">
-        <v>5.96</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="26">
@@ -46504,7 +46504,7 @@
         <v>3.3</v>
       </c>
       <c r="E26" t="n">
-        <v>4.06</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="27">
@@ -46518,10 +46518,10 @@
         <v>2</v>
       </c>
       <c r="D27" t="n">
-        <v>4.06</v>
+        <v>3.7</v>
       </c>
       <c r="E27" t="n">
-        <v>4.82</v>
+        <v>4.1</v>
       </c>
     </row>
     <row r="28">
@@ -46535,10 +46535,10 @@
         <v>1</v>
       </c>
       <c r="D28" t="n">
-        <v>4.82</v>
+        <v>4.1</v>
       </c>
       <c r="E28" t="n">
-        <v>5.2</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="29">
@@ -46555,7 +46555,7 @@
         <v>3.3</v>
       </c>
       <c r="E29" t="n">
-        <v>4.06</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="30">
@@ -46569,10 +46569,10 @@
         <v>2</v>
       </c>
       <c r="D30" t="n">
-        <v>4.06</v>
+        <v>3.7</v>
       </c>
       <c r="E30" t="n">
-        <v>4.82</v>
+        <v>4.1</v>
       </c>
     </row>
     <row r="31">
@@ -46586,10 +46586,10 @@
         <v>1</v>
       </c>
       <c r="D31" t="n">
-        <v>4.82</v>
+        <v>4.1</v>
       </c>
       <c r="E31" t="n">
-        <v>5.2</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="32">
@@ -46606,7 +46606,7 @@
         <v>3.3</v>
       </c>
       <c r="E32" t="n">
-        <v>3.68</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="33">
@@ -46620,10 +46620,10 @@
         <v>1</v>
       </c>
       <c r="D33" t="n">
-        <v>3.68</v>
+        <v>3.5</v>
       </c>
       <c r="E33" t="n">
-        <v>4.06</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="34">
@@ -46640,7 +46640,7 @@
         <v>3.3</v>
       </c>
       <c r="E34" t="n">
-        <v>5.96</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="35">
@@ -46654,10 +46654,10 @@
         <v>4</v>
       </c>
       <c r="D35" t="n">
-        <v>5.96</v>
+        <v>4.7</v>
       </c>
       <c r="E35" t="n">
-        <v>7.48</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="36">
@@ -46674,7 +46674,7 @@
         <v>3.3</v>
       </c>
       <c r="E36" t="n">
-        <v>5.58</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="37">
@@ -46688,10 +46688,10 @@
         <v>2</v>
       </c>
       <c r="D37" t="n">
-        <v>5.58</v>
+        <v>4.5</v>
       </c>
       <c r="E37" t="n">
-        <v>6.34</v>
+        <v>4.9</v>
       </c>
     </row>
     <row r="38">
@@ -46708,7 +46708,7 @@
         <v>3.3</v>
       </c>
       <c r="E38" t="n">
-        <v>5.2</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="39">
@@ -46722,10 +46722,10 @@
         <v>2</v>
       </c>
       <c r="D39" t="n">
-        <v>5.2</v>
+        <v>4.3</v>
       </c>
       <c r="E39" t="n">
-        <v>5.96</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="40">
@@ -46742,7 +46742,7 @@
         <v>3.3</v>
       </c>
       <c r="E40" t="n">
-        <v>5.2</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="41">
@@ -46756,10 +46756,10 @@
         <v>4</v>
       </c>
       <c r="D41" t="n">
-        <v>5.2</v>
+        <v>4.3</v>
       </c>
       <c r="E41" t="n">
-        <v>6.72</v>
+        <v>5.1</v>
       </c>
     </row>
     <row r="42">
@@ -46773,10 +46773,10 @@
         <v>4</v>
       </c>
       <c r="D42" t="n">
-        <v>6.72</v>
+        <v>5.1</v>
       </c>
       <c r="E42" t="n">
-        <v>8.24</v>
+        <v>5.9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
F04/F05 panel B: shrink F04 plot, add quadrant key below panel B
- F04: shift panel B 5mm left, narrow to 181mm (plot.margin tightened
  to keep panel A clear of overlap and bg stripes within figure)
- F04 + F05: add horizontal quadrant key below panel B (bg box +
  inner bar + label), 3rd item nudged right (Discordant ~3.6mm,
  Non-reversed ~1.8mm) to balance label spacing
- Engine: bg_extend_right cfg knob (default 2.0); F05 sets 0.05 so
  pathway bg stripes stop at X_BAR_MAX
- Box: F04/F05 main composites and S08/S09 supplementary xlsx synced
</commit_message>
<xml_diff>
--- a/04_Figures/F04/c_data/F04_supplementary.xlsx
+++ b/04_Figures/F04/c_data/F04_supplementary.xlsx
@@ -46096,7 +46096,7 @@
         <v>3.3</v>
       </c>
       <c r="E2" t="n">
-        <v>4.1</v>
+        <v>5.14</v>
       </c>
     </row>
     <row r="3">
@@ -46110,10 +46110,10 @@
         <v>3</v>
       </c>
       <c r="D3" t="n">
-        <v>4.1</v>
+        <v>5.14</v>
       </c>
       <c r="E3" t="n">
-        <v>4.7</v>
+        <v>6.52</v>
       </c>
     </row>
     <row r="4">
@@ -46127,10 +46127,10 @@
         <v>1</v>
       </c>
       <c r="D4" t="n">
-        <v>4.7</v>
+        <v>6.52</v>
       </c>
       <c r="E4" t="n">
-        <v>4.9</v>
+        <v>6.98</v>
       </c>
     </row>
     <row r="5">
@@ -46147,7 +46147,7 @@
         <v>3.3</v>
       </c>
       <c r="E5" t="n">
-        <v>4.1</v>
+        <v>5.14</v>
       </c>
     </row>
     <row r="6">
@@ -46161,10 +46161,10 @@
         <v>2</v>
       </c>
       <c r="D6" t="n">
-        <v>4.1</v>
+        <v>5.14</v>
       </c>
       <c r="E6" t="n">
-        <v>4.5</v>
+        <v>6.06</v>
       </c>
     </row>
     <row r="7">
@@ -46178,10 +46178,10 @@
         <v>1</v>
       </c>
       <c r="D7" t="n">
-        <v>4.5</v>
+        <v>6.06</v>
       </c>
       <c r="E7" t="n">
-        <v>4.7</v>
+        <v>6.52</v>
       </c>
     </row>
     <row r="8">
@@ -46198,7 +46198,7 @@
         <v>3.3</v>
       </c>
       <c r="E8" t="n">
-        <v>3.7</v>
+        <v>4.22</v>
       </c>
     </row>
     <row r="9">
@@ -46212,10 +46212,10 @@
         <v>2</v>
       </c>
       <c r="D9" t="n">
-        <v>3.7</v>
+        <v>4.22</v>
       </c>
       <c r="E9" t="n">
-        <v>4.1</v>
+        <v>5.14</v>
       </c>
     </row>
     <row r="10">
@@ -46229,10 +46229,10 @@
         <v>1</v>
       </c>
       <c r="D10" t="n">
-        <v>4.1</v>
+        <v>5.14</v>
       </c>
       <c r="E10" t="n">
-        <v>4.3</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="11">
@@ -46249,7 +46249,7 @@
         <v>3.3</v>
       </c>
       <c r="E11" t="n">
-        <v>4.3</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="12">
@@ -46263,10 +46263,10 @@
         <v>2</v>
       </c>
       <c r="D12" t="n">
-        <v>4.3</v>
+        <v>5.6</v>
       </c>
       <c r="E12" t="n">
-        <v>4.7</v>
+        <v>6.52</v>
       </c>
     </row>
     <row r="13">
@@ -46280,10 +46280,10 @@
         <v>1</v>
       </c>
       <c r="D13" t="n">
-        <v>4.7</v>
+        <v>6.52</v>
       </c>
       <c r="E13" t="n">
-        <v>4.9</v>
+        <v>6.98</v>
       </c>
     </row>
     <row r="14">
@@ -46300,7 +46300,7 @@
         <v>3.3</v>
       </c>
       <c r="E14" t="n">
-        <v>4.3</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="15">
@@ -46314,10 +46314,10 @@
         <v>3</v>
       </c>
       <c r="D15" t="n">
-        <v>4.3</v>
+        <v>5.6</v>
       </c>
       <c r="E15" t="n">
-        <v>4.9</v>
+        <v>6.98</v>
       </c>
     </row>
     <row r="16">
@@ -46331,10 +46331,10 @@
         <v>2</v>
       </c>
       <c r="D16" t="n">
-        <v>4.9</v>
+        <v>6.98</v>
       </c>
       <c r="E16" t="n">
-        <v>5.3</v>
+        <v>7.9</v>
       </c>
     </row>
     <row r="17">
@@ -46351,7 +46351,7 @@
         <v>3.3</v>
       </c>
       <c r="E17" t="n">
-        <v>3.5</v>
+        <v>3.76</v>
       </c>
     </row>
     <row r="18">
@@ -46365,10 +46365,10 @@
         <v>1</v>
       </c>
       <c r="D18" t="n">
-        <v>3.5</v>
+        <v>3.76</v>
       </c>
       <c r="E18" t="n">
-        <v>3.7</v>
+        <v>4.22</v>
       </c>
     </row>
     <row r="19">
@@ -46382,10 +46382,10 @@
         <v>1</v>
       </c>
       <c r="D19" t="n">
-        <v>3.7</v>
+        <v>4.22</v>
       </c>
       <c r="E19" t="n">
-        <v>3.9</v>
+        <v>4.68</v>
       </c>
     </row>
     <row r="20">
@@ -46402,7 +46402,7 @@
         <v>3.3</v>
       </c>
       <c r="E20" t="n">
-        <v>4.3</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="21">
@@ -46416,10 +46416,10 @@
         <v>3</v>
       </c>
       <c r="D21" t="n">
-        <v>4.3</v>
+        <v>5.6</v>
       </c>
       <c r="E21" t="n">
-        <v>4.9</v>
+        <v>6.98</v>
       </c>
     </row>
     <row r="22">
@@ -46433,10 +46433,10 @@
         <v>1</v>
       </c>
       <c r="D22" t="n">
-        <v>4.9</v>
+        <v>6.98</v>
       </c>
       <c r="E22" t="n">
-        <v>5.1</v>
+        <v>7.44</v>
       </c>
     </row>
     <row r="23">
@@ -46453,7 +46453,7 @@
         <v>3.3</v>
       </c>
       <c r="E23" t="n">
-        <v>3.9</v>
+        <v>4.68</v>
       </c>
     </row>
     <row r="24">
@@ -46467,10 +46467,10 @@
         <v>3</v>
       </c>
       <c r="D24" t="n">
-        <v>3.9</v>
+        <v>4.68</v>
       </c>
       <c r="E24" t="n">
-        <v>4.5</v>
+        <v>6.06</v>
       </c>
     </row>
     <row r="25">
@@ -46484,10 +46484,10 @@
         <v>1</v>
       </c>
       <c r="D25" t="n">
-        <v>4.5</v>
+        <v>6.06</v>
       </c>
       <c r="E25" t="n">
-        <v>4.7</v>
+        <v>6.52</v>
       </c>
     </row>
     <row r="26">
@@ -46504,7 +46504,7 @@
         <v>3.3</v>
       </c>
       <c r="E26" t="n">
-        <v>3.7</v>
+        <v>4.22</v>
       </c>
     </row>
     <row r="27">
@@ -46518,10 +46518,10 @@
         <v>2</v>
       </c>
       <c r="D27" t="n">
-        <v>3.7</v>
+        <v>4.22</v>
       </c>
       <c r="E27" t="n">
-        <v>4.1</v>
+        <v>5.14</v>
       </c>
     </row>
     <row r="28">
@@ -46535,10 +46535,10 @@
         <v>1</v>
       </c>
       <c r="D28" t="n">
-        <v>4.1</v>
+        <v>5.14</v>
       </c>
       <c r="E28" t="n">
-        <v>4.3</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="29">
@@ -46555,7 +46555,7 @@
         <v>3.3</v>
       </c>
       <c r="E29" t="n">
-        <v>3.7</v>
+        <v>4.22</v>
       </c>
     </row>
     <row r="30">
@@ -46569,10 +46569,10 @@
         <v>2</v>
       </c>
       <c r="D30" t="n">
-        <v>3.7</v>
+        <v>4.22</v>
       </c>
       <c r="E30" t="n">
-        <v>4.1</v>
+        <v>5.14</v>
       </c>
     </row>
     <row r="31">
@@ -46586,10 +46586,10 @@
         <v>1</v>
       </c>
       <c r="D31" t="n">
-        <v>4.1</v>
+        <v>5.14</v>
       </c>
       <c r="E31" t="n">
-        <v>4.3</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="32">
@@ -46606,7 +46606,7 @@
         <v>3.3</v>
       </c>
       <c r="E32" t="n">
-        <v>3.5</v>
+        <v>3.76</v>
       </c>
     </row>
     <row r="33">
@@ -46620,10 +46620,10 @@
         <v>1</v>
       </c>
       <c r="D33" t="n">
-        <v>3.5</v>
+        <v>3.76</v>
       </c>
       <c r="E33" t="n">
-        <v>3.7</v>
+        <v>4.22</v>
       </c>
     </row>
     <row r="34">
@@ -46640,7 +46640,7 @@
         <v>3.3</v>
       </c>
       <c r="E34" t="n">
-        <v>4.7</v>
+        <v>6.52</v>
       </c>
     </row>
     <row r="35">
@@ -46654,10 +46654,10 @@
         <v>4</v>
       </c>
       <c r="D35" t="n">
-        <v>4.7</v>
+        <v>6.52</v>
       </c>
       <c r="E35" t="n">
-        <v>5.5</v>
+        <v>8.36</v>
       </c>
     </row>
     <row r="36">
@@ -46674,7 +46674,7 @@
         <v>3.3</v>
       </c>
       <c r="E36" t="n">
-        <v>4.5</v>
+        <v>6.06</v>
       </c>
     </row>
     <row r="37">
@@ -46688,10 +46688,10 @@
         <v>2</v>
       </c>
       <c r="D37" t="n">
-        <v>4.5</v>
+        <v>6.06</v>
       </c>
       <c r="E37" t="n">
-        <v>4.9</v>
+        <v>6.98</v>
       </c>
     </row>
     <row r="38">
@@ -46708,7 +46708,7 @@
         <v>3.3</v>
       </c>
       <c r="E38" t="n">
-        <v>4.3</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="39">
@@ -46722,10 +46722,10 @@
         <v>2</v>
       </c>
       <c r="D39" t="n">
-        <v>4.3</v>
+        <v>5.6</v>
       </c>
       <c r="E39" t="n">
-        <v>4.7</v>
+        <v>6.52</v>
       </c>
     </row>
     <row r="40">
@@ -46742,7 +46742,7 @@
         <v>3.3</v>
       </c>
       <c r="E40" t="n">
-        <v>4.3</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="41">
@@ -46756,10 +46756,10 @@
         <v>4</v>
       </c>
       <c r="D41" t="n">
-        <v>4.3</v>
+        <v>5.6</v>
       </c>
       <c r="E41" t="n">
-        <v>5.1</v>
+        <v>7.44</v>
       </c>
     </row>
     <row r="42">
@@ -46773,10 +46773,10 @@
         <v>4</v>
       </c>
       <c r="D42" t="n">
-        <v>5.1</v>
+        <v>7.44</v>
       </c>
       <c r="E42" t="n">
-        <v>5.9</v>
+        <v>9.28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
refactor(F02-F05): tighten panel scripts and regenerate outputs
- Drop redundant section-header comments and unused intermediates
  across F02, F03, F04, F05 main + supp panel scripts.
- Regenerate all composite figures and supplementary xlsx workbooks
  to match the tightened scripts.
</commit_message>
<xml_diff>
--- a/04_Figures/F04/c_data/F04_supplementary.xlsx
+++ b/04_Figures/F04/c_data/F04_supplementary.xlsx
@@ -36258,25 +36258,25 @@
         <v>218</v>
       </c>
       <c r="D2" t="n">
-        <v>3.48412721247129</v>
+        <v>3.48412721247115</v>
       </c>
       <c r="E2" t="n">
-        <v>4.21161096897919</v>
+        <v>4.21161096897894</v>
       </c>
       <c r="F2" t="n">
         <v>0.511141040596115</v>
       </c>
       <c r="G2" t="n">
-        <v>0.556196949731639</v>
+        <v>0.556196949731628</v>
       </c>
       <c r="H2" t="n">
-        <v>0.0287632004854532</v>
+        <v>0.0287632004854626</v>
       </c>
       <c r="I2" t="s">
         <v>219</v>
       </c>
       <c r="J2" t="n">
-        <v>4.21161096897919</v>
+        <v>4.21161096897894</v>
       </c>
       <c r="K2" t="s">
         <v>15</v>
@@ -36293,25 +36293,25 @@
         <v>218</v>
       </c>
       <c r="D3" t="n">
-        <v>4.05790561093415</v>
+        <v>4.05790561093385</v>
       </c>
       <c r="E3" t="n">
-        <v>4.09186896159768</v>
+        <v>4.09186896159723</v>
       </c>
       <c r="F3" t="n">
-        <v>0.706915668807518</v>
+        <v>0.706915668807515</v>
       </c>
       <c r="G3" t="n">
-        <v>0.64771515727271</v>
+        <v>0.647715157272685</v>
       </c>
       <c r="H3" t="n">
-        <v>0.00213423371891747</v>
+        <v>0.00213423371891966</v>
       </c>
       <c r="I3" t="s">
         <v>219</v>
       </c>
       <c r="J3" t="n">
-        <v>4.09186896159768</v>
+        <v>4.09186896159723</v>
       </c>
       <c r="K3" t="s">
         <v>15</v>
@@ -36328,25 +36328,25 @@
         <v>220</v>
       </c>
       <c r="D4" t="n">
-        <v>-3.4881722003434</v>
+        <v>-3.48817220034292</v>
       </c>
       <c r="E4" t="n">
-        <v>-3.45429041055465</v>
+        <v>-3.45429041055405</v>
       </c>
       <c r="F4" t="n">
-        <v>-0.764142564725148</v>
+        <v>-0.764142564725137</v>
       </c>
       <c r="G4" t="n">
-        <v>-0.739464072659462</v>
+        <v>-0.739464072659423</v>
       </c>
       <c r="H4" t="n">
-        <v>0.00480638078838799</v>
+        <v>0.00480638078839455</v>
       </c>
       <c r="I4" t="s">
         <v>221</v>
       </c>
       <c r="J4" t="n">
-        <v>3.45429041055465</v>
+        <v>3.45429041055405</v>
       </c>
       <c r="K4" t="s">
         <v>39</v>
@@ -36363,25 +36363,25 @@
         <v>218</v>
       </c>
       <c r="D5" t="n">
-        <v>2.59704840828289</v>
+        <v>2.5970484082824</v>
       </c>
       <c r="E5" t="n">
-        <v>3.43072370614807</v>
+        <v>3.43072370614742</v>
       </c>
       <c r="F5" t="n">
         <v>1.10652955402938</v>
       </c>
       <c r="G5" t="n">
-        <v>1.71883830144357</v>
+        <v>1.71883830144356</v>
       </c>
       <c r="H5" t="n">
-        <v>0.00758883678460189</v>
+        <v>0.00758883678461347</v>
       </c>
       <c r="I5" t="s">
         <v>219</v>
       </c>
       <c r="J5" t="n">
-        <v>3.43072370614807</v>
+        <v>3.43072370614742</v>
       </c>
       <c r="K5" t="s">
         <v>15</v>
@@ -36398,25 +36398,25 @@
         <v>220</v>
       </c>
       <c r="D6" t="n">
-        <v>-4.64310062264231</v>
+        <v>-4.6431006226425</v>
       </c>
       <c r="E6" t="n">
-        <v>-2.91801758322959</v>
+        <v>-2.91801758322966</v>
       </c>
       <c r="F6" t="n">
-        <v>-0.481424194198411</v>
+        <v>-0.481424194198414</v>
       </c>
       <c r="G6" t="n">
-        <v>-0.309755822129894</v>
+        <v>-0.30975582212989</v>
       </c>
       <c r="H6" t="n">
-        <v>0.00523848038285758</v>
+        <v>0.00523848038285679</v>
       </c>
       <c r="I6" t="s">
         <v>221</v>
       </c>
       <c r="J6" t="n">
-        <v>2.91801758322959</v>
+        <v>2.91801758322966</v>
       </c>
       <c r="K6" t="s">
         <v>39</v>
@@ -36433,25 +36433,25 @@
         <v>218</v>
       </c>
       <c r="D7" t="n">
-        <v>3.76368067195992</v>
+        <v>3.76368067196001</v>
       </c>
       <c r="E7" t="n">
-        <v>2.88994882485869</v>
+        <v>2.88994882485905</v>
       </c>
       <c r="F7" t="n">
-        <v>0.390491085452172</v>
+        <v>0.390491085452169</v>
       </c>
       <c r="G7" t="n">
-        <v>0.306973060642743</v>
+        <v>0.306973060642772</v>
       </c>
       <c r="H7" t="n">
-        <v>0.0458883291390259</v>
+        <v>0.045888329139026</v>
       </c>
       <c r="I7" t="s">
         <v>219</v>
       </c>
       <c r="J7" t="n">
-        <v>2.88994882485869</v>
+        <v>2.88994882485905</v>
       </c>
       <c r="K7" t="s">
         <v>15</v>
@@ -36468,25 +36468,25 @@
         <v>218</v>
       </c>
       <c r="D8" t="n">
-        <v>4.6362501064832</v>
+        <v>4.63625010648391</v>
       </c>
       <c r="E8" t="n">
-        <v>2.88766399959219</v>
+        <v>2.88766399959269</v>
       </c>
       <c r="F8" t="n">
-        <v>0.433831594366477</v>
+        <v>0.433831594366481</v>
       </c>
       <c r="G8" t="n">
-        <v>0.25369598668917</v>
+        <v>0.253695986689177</v>
       </c>
       <c r="H8" t="n">
-        <v>0.00936752333385777</v>
+        <v>0.00936752333384944</v>
       </c>
       <c r="I8" t="s">
         <v>219</v>
       </c>
       <c r="J8" t="n">
-        <v>2.88766399959219</v>
+        <v>2.88766399959269</v>
       </c>
       <c r="K8" t="s">
         <v>15</v>
@@ -36503,25 +36503,25 @@
         <v>218</v>
       </c>
       <c r="D9" t="n">
-        <v>5.39120431822591</v>
+        <v>5.39120431822665</v>
       </c>
       <c r="E9" t="n">
-        <v>2.75946428310965</v>
+        <v>2.75946428311011</v>
       </c>
       <c r="F9" t="n">
-        <v>0.473425956401492</v>
+        <v>0.473425956401499</v>
       </c>
       <c r="G9" t="n">
-        <v>0.248086314903833</v>
+        <v>0.248086314903844</v>
       </c>
       <c r="H9" t="n">
-        <v>0.00154451475019621</v>
+        <v>0.00154451475019456</v>
       </c>
       <c r="I9" t="s">
         <v>219</v>
       </c>
       <c r="J9" t="n">
-        <v>2.75946428310965</v>
+        <v>2.75946428311011</v>
       </c>
       <c r="K9" t="s">
         <v>15</v>
@@ -36538,25 +36538,25 @@
         <v>220</v>
       </c>
       <c r="D10" t="n">
-        <v>-3.20564732472382</v>
+        <v>-3.20564732472344</v>
       </c>
       <c r="E10" t="n">
-        <v>-2.70712786773453</v>
+        <v>-2.70712786773419</v>
       </c>
       <c r="F10" t="n">
-        <v>-0.814653105627787</v>
+        <v>-0.814653105627801</v>
       </c>
       <c r="G10" t="n">
-        <v>-0.693627278270892</v>
+        <v>-0.693627278270899</v>
       </c>
       <c r="H10" t="n">
-        <v>0.006699503612022</v>
+        <v>0.00669950361202838</v>
       </c>
       <c r="I10" t="s">
         <v>221</v>
       </c>
       <c r="J10" t="n">
-        <v>2.70712786773453</v>
+        <v>2.70712786773419</v>
       </c>
       <c r="K10" t="s">
         <v>39</v>
@@ -36573,25 +36573,25 @@
         <v>218</v>
       </c>
       <c r="D11" t="n">
-        <v>4.62111071584404</v>
+        <v>4.62111071584342</v>
       </c>
       <c r="E11" t="n">
-        <v>2.67928195405153</v>
+        <v>2.67928195405119</v>
       </c>
       <c r="F11" t="n">
-        <v>1.11357792651978</v>
+        <v>1.11357792651977</v>
       </c>
       <c r="G11" t="n">
-        <v>0.661004499617036</v>
+        <v>0.66100449961704</v>
       </c>
       <c r="H11" t="n">
-        <v>0.00000578698121710783</v>
+        <v>0.00000578698121712521</v>
       </c>
       <c r="I11" t="s">
         <v>219</v>
       </c>
       <c r="J11" t="n">
-        <v>2.67928195405153</v>
+        <v>2.67928195405119</v>
       </c>
       <c r="K11" t="s">
         <v>15</v>
@@ -36608,25 +36608,25 @@
         <v>220</v>
       </c>
       <c r="D12" t="n">
-        <v>-2.91392784946499</v>
+        <v>-2.91392784946468</v>
       </c>
       <c r="E12" t="n">
-        <v>-2.46744007168027</v>
+        <v>-2.46744007167997</v>
       </c>
       <c r="F12" t="n">
-        <v>-0.60829357813018</v>
+        <v>-0.608293578130183</v>
       </c>
       <c r="G12" t="n">
-        <v>-0.441667173414011</v>
+        <v>-0.441667173414007</v>
       </c>
       <c r="H12" t="n">
-        <v>0.0423994348400474</v>
+        <v>0.0423994348400729</v>
       </c>
       <c r="I12" t="s">
         <v>221</v>
       </c>
       <c r="J12" t="n">
-        <v>2.46744007168027</v>
+        <v>2.46744007167997</v>
       </c>
       <c r="K12" t="s">
         <v>39</v>
@@ -36643,25 +36643,25 @@
         <v>218</v>
       </c>
       <c r="D13" t="n">
-        <v>3.56494917113622</v>
+        <v>3.56494917113591</v>
       </c>
       <c r="E13" t="n">
-        <v>2.43367358253536</v>
+        <v>2.4336735825353</v>
       </c>
       <c r="F13" t="n">
-        <v>0.538929847075678</v>
+        <v>0.538929847075671</v>
       </c>
       <c r="G13" t="n">
-        <v>0.376663015654117</v>
+        <v>0.376663015654135</v>
       </c>
       <c r="H13" t="n">
-        <v>0.0200502138750984</v>
+        <v>0.0200502138751121</v>
       </c>
       <c r="I13" t="s">
         <v>219</v>
       </c>
       <c r="J13" t="n">
-        <v>2.43367358253536</v>
+        <v>2.4336735825353</v>
       </c>
       <c r="K13" t="s">
         <v>15</v>
@@ -36678,25 +36678,25 @@
         <v>220</v>
       </c>
       <c r="D14" t="n">
-        <v>-4.18249954175594</v>
+        <v>-4.18249954175544</v>
       </c>
       <c r="E14" t="n">
-        <v>-2.37026507714442</v>
+        <v>-2.37026507714425</v>
       </c>
       <c r="F14" t="n">
-        <v>-0.769667406399481</v>
+        <v>-0.769667406399471</v>
       </c>
       <c r="G14" t="n">
-        <v>-0.431402455948788</v>
+        <v>-0.431402455948803</v>
       </c>
       <c r="H14" t="n">
-        <v>0.00080391981779155</v>
+        <v>0.00080391981779289</v>
       </c>
       <c r="I14" t="s">
         <v>221</v>
       </c>
       <c r="J14" t="n">
-        <v>2.37026507714442</v>
+        <v>2.37026507714425</v>
       </c>
       <c r="K14" t="s">
         <v>39</v>
@@ -36713,25 +36713,25 @@
         <v>218</v>
       </c>
       <c r="D15" t="n">
-        <v>3.25356019722925</v>
+        <v>3.25356019722879</v>
       </c>
       <c r="E15" t="n">
-        <v>2.32286999909631</v>
+        <v>2.32286999909601</v>
       </c>
       <c r="F15" t="n">
-        <v>0.900404254930407</v>
+        <v>0.900404254930406</v>
       </c>
       <c r="G15" t="n">
-        <v>0.413709003406987</v>
+        <v>0.413709003406991</v>
       </c>
       <c r="H15" t="n">
-        <v>0.00466372750746012</v>
+        <v>0.00466372750746704</v>
       </c>
       <c r="I15" t="s">
         <v>219</v>
       </c>
       <c r="J15" t="n">
-        <v>2.32286999909631</v>
+        <v>2.32286999909601</v>
       </c>
       <c r="K15" t="s">
         <v>15</v>
@@ -36748,25 +36748,25 @@
         <v>218</v>
       </c>
       <c r="D16" t="n">
-        <v>4.0178573046977</v>
+        <v>4.01785730469785</v>
       </c>
       <c r="E16" t="n">
-        <v>2.29300875076201</v>
+        <v>2.2930087507622</v>
       </c>
       <c r="F16" t="n">
-        <v>0.402624473620968</v>
+        <v>0.402624473620961</v>
       </c>
       <c r="G16" t="n">
-        <v>0.235246478227104</v>
+        <v>0.235246478227111</v>
       </c>
       <c r="H16" t="n">
-        <v>0.0297225836246233</v>
+        <v>0.0297225836246227</v>
       </c>
       <c r="I16" t="s">
         <v>219</v>
       </c>
       <c r="J16" t="n">
-        <v>2.29300875076201</v>
+        <v>2.2930087507622</v>
       </c>
       <c r="K16" t="s">
         <v>15</v>
@@ -36783,25 +36783,25 @@
         <v>218</v>
       </c>
       <c r="D17" t="n">
-        <v>3.98464356645387</v>
+        <v>3.9846435664542</v>
       </c>
       <c r="E17" t="n">
-        <v>2.25856204382237</v>
+        <v>2.2585620438228</v>
       </c>
       <c r="F17" t="n">
-        <v>0.349460320731534</v>
+        <v>0.34946032073152</v>
       </c>
       <c r="G17" t="n">
-        <v>0.2027926331901</v>
+        <v>0.202792633190114</v>
       </c>
       <c r="H17" t="n">
-        <v>0.0491609257512415</v>
+        <v>0.049160925751234</v>
       </c>
       <c r="I17" t="s">
         <v>219</v>
       </c>
       <c r="J17" t="n">
-        <v>2.25856204382237</v>
+        <v>2.2585620438228</v>
       </c>
       <c r="K17" t="s">
         <v>15</v>
@@ -36818,25 +36818,25 @@
         <v>218</v>
       </c>
       <c r="D18" t="n">
-        <v>3.73354463132545</v>
+        <v>3.73354463132493</v>
       </c>
       <c r="E18" t="n">
-        <v>2.13914502585476</v>
+        <v>2.13914502585422</v>
       </c>
       <c r="F18" t="n">
-        <v>0.776205944356491</v>
+        <v>0.776205944356487</v>
       </c>
       <c r="G18" t="n">
-        <v>0.452181538535665</v>
+        <v>0.452181538535612</v>
       </c>
       <c r="H18" t="n">
-        <v>0.0025772311745655</v>
+        <v>0.00257723117456945</v>
       </c>
       <c r="I18" t="s">
         <v>219</v>
       </c>
       <c r="J18" t="n">
-        <v>2.13914502585476</v>
+        <v>2.13914502585422</v>
       </c>
       <c r="K18" t="s">
         <v>15</v>
@@ -36853,25 +36853,25 @@
         <v>218</v>
       </c>
       <c r="D19" t="n">
-        <v>3.9078914232885</v>
+        <v>3.90789142328831</v>
       </c>
       <c r="E19" t="n">
-        <v>2.02585547110802</v>
+        <v>2.02585547110797</v>
       </c>
       <c r="F19" t="n">
-        <v>0.611262057913596</v>
+        <v>0.611262057913599</v>
       </c>
       <c r="G19" t="n">
-        <v>0.285039023149757</v>
+        <v>0.285039023149764</v>
       </c>
       <c r="H19" t="n">
-        <v>0.00639334703822732</v>
+        <v>0.00639334703823077</v>
       </c>
       <c r="I19" t="s">
         <v>219</v>
       </c>
       <c r="J19" t="n">
-        <v>2.02585547110802</v>
+        <v>2.02585547110797</v>
       </c>
       <c r="K19" t="s">
         <v>15</v>
@@ -36888,25 +36888,25 @@
         <v>218</v>
       </c>
       <c r="D20" t="n">
-        <v>4.63999909161819</v>
+        <v>4.63999909161752</v>
       </c>
       <c r="E20" t="n">
-        <v>1.95027028471445</v>
+        <v>1.95027028471429</v>
       </c>
       <c r="F20" t="n">
-        <v>1.01770635395492</v>
+        <v>1.0177063539549</v>
       </c>
       <c r="G20" t="n">
-        <v>0.437936508011408</v>
+        <v>0.437936508011425</v>
       </c>
       <c r="H20" t="n">
-        <v>0.0000152558240329967</v>
+        <v>0.0000152558240330445</v>
       </c>
       <c r="I20" t="s">
         <v>219</v>
       </c>
       <c r="J20" t="n">
-        <v>1.95027028471445</v>
+        <v>1.95027028471429</v>
       </c>
       <c r="K20" t="s">
         <v>15</v>
@@ -36923,25 +36923,25 @@
         <v>218</v>
       </c>
       <c r="D21" t="n">
-        <v>4.98144460589381</v>
+        <v>4.98144460589374</v>
       </c>
       <c r="E21" t="n">
-        <v>1.94065606360796</v>
+        <v>1.94065606360806</v>
       </c>
       <c r="F21" t="n">
-        <v>0.540644965102565</v>
+        <v>0.540644965102548</v>
       </c>
       <c r="G21" t="n">
-        <v>0.21563397466149</v>
+        <v>0.215633974661497</v>
       </c>
       <c r="H21" t="n">
-        <v>0.00141070927441336</v>
+        <v>0.00141070927441428</v>
       </c>
       <c r="I21" t="s">
         <v>219</v>
       </c>
       <c r="J21" t="n">
-        <v>1.94065606360796</v>
+        <v>1.94065606360806</v>
       </c>
       <c r="K21" t="s">
         <v>15</v>

</xml_diff>